<commit_message>
feat: Export PR as PDF but not identical as the offical PR form
</commit_message>
<xml_diff>
--- a/procurement_documents/Purchase Request Excel Template.xlsx
+++ b/procurement_documents/Purchase Request Excel Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9B3A2A2-6D2D-4D6D-AC8E-2C23045E595F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC4A4F9-6522-48F8-BEA2-B27FF43D7476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="947" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
   <si>
     <t>Department:</t>
   </si>
@@ -123,12 +123,6 @@
   </si>
   <si>
     <t>pr_date</t>
-  </si>
-  <si>
-    <t>pr_name_of_request     pr_approved_by (user_fullname FIRST NAME M.I SURNAME format)</t>
-  </si>
-  <si>
-    <t>pr_designation                                             pr_approved_by_designation</t>
   </si>
   <si>
     <t>pr_purpose</t>
@@ -161,7 +155,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy;@"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,13 +303,6 @@
       <color theme="1"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="20"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10.5"/>
@@ -352,7 +339,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -400,16 +387,95 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
@@ -418,127 +484,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -561,20 +506,20 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
@@ -591,22 +536,154 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -620,47 +697,16 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
@@ -672,126 +718,9 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -802,23 +731,31 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -828,19 +765,6 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -859,7 +783,7 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -880,9 +804,9 @@
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -911,26 +835,23 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -938,228 +859,205 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="2" borderId="40" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="2" borderId="28" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="39" fontId="27" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="39" fontId="26" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="22" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="22" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1708,8 +1606,7 @@
   <cols>
     <col min="1" max="1" width="10.28515625" style="3" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="10" style="3" customWidth="1"/>
-    <col min="4" max="4" width="48.7109375" style="3" customWidth="1"/>
+    <col min="3" max="4" width="29.28515625" style="3" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" style="3" customWidth="1"/>
     <col min="6" max="6" width="6.140625" style="3" customWidth="1"/>
     <col min="7" max="7" width="19.85546875" style="3" customWidth="1"/>
@@ -1718,164 +1615,164 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="25"/>
-    </row>
-    <row r="2" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="22"/>
+    </row>
+    <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16"/>
-      <c r="B2" s="92" t="s">
+      <c r="B2" s="88" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="92"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="94" t="s">
+      <c r="C2" s="88"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="92"/>
-      <c r="G2" s="95"/>
-    </row>
-    <row r="3" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F2" s="94"/>
+      <c r="G2" s="89"/>
+    </row>
+    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="17"/>
-      <c r="B3" s="96" t="s">
+      <c r="B3" s="90" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="96"/>
-      <c r="D3" s="97"/>
-      <c r="E3" s="98" t="s">
+      <c r="C3" s="90"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="99"/>
-      <c r="G3" s="100"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="58"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="16"/>
-      <c r="B4" s="92" t="s">
+      <c r="B4" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="92"/>
-      <c r="D4" s="93"/>
-      <c r="E4" s="101"/>
-      <c r="F4" s="102"/>
-      <c r="G4" s="100"/>
-    </row>
-    <row r="5" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C4" s="88"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="58"/>
+    </row>
+    <row r="5" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="17"/>
-      <c r="B5" s="87" t="s">
+      <c r="B5" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="87"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="89" t="s">
+      <c r="C5" s="92"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="90"/>
-      <c r="G5" s="91"/>
-    </row>
-    <row r="6" spans="1:14" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="26"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="30"/>
-    </row>
-    <row r="7" spans="1:14" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="19"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-    </row>
-    <row r="8" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="32" t="s">
+      <c r="F5" s="30"/>
+      <c r="G5" s="31"/>
+    </row>
+    <row r="6" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="23"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="25"/>
+    </row>
+    <row r="7" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+    </row>
+    <row r="8" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="78" t="s">
+      <c r="B8" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="78"/>
-      <c r="D8" s="79"/>
-      <c r="E8" s="18" t="s">
+      <c r="C8" s="80"/>
+      <c r="D8" s="81"/>
+      <c r="E8" s="82" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="103" t="s">
+      <c r="F8" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="104"/>
+      <c r="G8" s="84"/>
       <c r="H8" s="4"/>
     </row>
-    <row r="9" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+    <row r="9" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="78" t="s">
+      <c r="B9" s="80" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="78"/>
-      <c r="D9" s="79"/>
-      <c r="E9" s="31" t="s">
+      <c r="C9" s="80"/>
+      <c r="D9" s="81"/>
+      <c r="E9" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="80" t="s">
+      <c r="F9" s="86" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="81"/>
+      <c r="G9" s="87"/>
     </row>
     <row r="10" spans="1:14" ht="8.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="82"/>
-      <c r="B10" s="83"/>
-      <c r="C10" s="83"/>
-      <c r="D10" s="83"/>
-      <c r="E10" s="83"/>
-      <c r="F10" s="83"/>
-      <c r="G10" s="83"/>
+      <c r="A10" s="35"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="84" t="s">
+      <c r="C11" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="85"/>
-      <c r="E11" s="84" t="s">
+      <c r="D11" s="38"/>
+      <c r="E11" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="86"/>
-      <c r="G11" s="34" t="s">
+      <c r="F11" s="39"/>
+      <c r="G11" s="27" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="D12" s="33"/>
+      <c r="E12" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="76" t="s">
+      <c r="F12" s="34"/>
+      <c r="G12" s="28" t="s">
         <v>34</v>
-      </c>
-      <c r="D12" s="77"/>
-      <c r="E12" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="35" t="s">
-        <v>36</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -1887,21 +1784,21 @@
     </row>
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="D13" s="33"/>
+      <c r="E13" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="76" t="s">
+      <c r="F13" s="34"/>
+      <c r="G13" s="28" t="s">
         <v>34</v>
-      </c>
-      <c r="D13" s="77"/>
-      <c r="E13" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="39"/>
-      <c r="G13" s="35" t="s">
-        <v>36</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -1912,456 +1809,426 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="76"/>
-      <c r="D14" s="77"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="35"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="28"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="76"/>
-      <c r="D15" s="77"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="35"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="28"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="76"/>
-      <c r="D16" s="77"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="35"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="28"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="76"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="35"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="28"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="35"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="28"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="35"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="28"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="35"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="28"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="35"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="28"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="35"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="28"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="35"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="28"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="35"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="28"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="35"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="28"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="35"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="28"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="35"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="28"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="73"/>
-      <c r="D28" s="74"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="35"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="28"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="73"/>
-      <c r="D29" s="75"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="35"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="28"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="73"/>
-      <c r="D30" s="74"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="35"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="28"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="37"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
-      <c r="G31" s="35"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="28"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="37"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="35"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="28"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="35"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="28"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="37"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="35"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="28"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
-      <c r="G35" s="35"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="28"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="37"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="35"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="28"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="38"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="39"/>
-      <c r="G37" s="35"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="28"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="35"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="28"/>
       <c r="H38" s="10"/>
     </row>
-    <row r="39" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="69"/>
-      <c r="D39" s="70"/>
-      <c r="E39" s="71"/>
-      <c r="F39" s="72"/>
-      <c r="G39" s="35"/>
+      <c r="C39" s="45"/>
+      <c r="D39" s="46"/>
+      <c r="E39" s="47"/>
+      <c r="F39" s="48"/>
+      <c r="G39" s="28"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="39"/>
-      <c r="G40" s="35"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="34"/>
+      <c r="F40" s="34"/>
+      <c r="G40" s="28"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="39"/>
-      <c r="F41" s="39"/>
-      <c r="G41" s="35"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="34"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="28"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="37"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="39"/>
-      <c r="G42" s="35"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="34"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="28"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="38"/>
-      <c r="E43" s="39"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="35"/>
+      <c r="C43" s="40"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="34"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="28"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="37"/>
-      <c r="D44" s="38"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="35"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="41"/>
+      <c r="E44" s="34"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="28"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14"/>
       <c r="B45" s="15"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="41"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
-      <c r="G45" s="35"/>
+      <c r="C45" s="50"/>
+      <c r="D45" s="51"/>
+      <c r="E45" s="34"/>
+      <c r="F45" s="34"/>
+      <c r="G45" s="28"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="42" t="s">
+      <c r="A46" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="B46" s="43"/>
-      <c r="C46" s="43"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="44"/>
-      <c r="F46" s="45" t="s">
-        <v>37</v>
-      </c>
-      <c r="G46" s="46"/>
+      <c r="B46" s="53"/>
+      <c r="C46" s="53"/>
+      <c r="D46" s="53"/>
+      <c r="E46" s="54"/>
+      <c r="F46" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="G46" s="56"/>
       <c r="H46" s="10"/>
     </row>
-    <row r="47" spans="1:8" ht="8.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="53"/>
-      <c r="B47" s="54"/>
-      <c r="C47" s="54"/>
-      <c r="D47" s="54"/>
-      <c r="E47" s="54"/>
-      <c r="F47" s="54"/>
-      <c r="G47" s="54"/>
-    </row>
-    <row r="48" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="55" t="s">
+    <row r="47" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="59"/>
+      <c r="B47" s="60"/>
+      <c r="C47" s="60"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="60"/>
+      <c r="F47" s="60"/>
+      <c r="G47" s="60"/>
+    </row>
+    <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="65" t="s">
         <v>24</v>
       </c>
-      <c r="B48" s="56"/>
-      <c r="C48" s="57" t="s">
-        <v>31</v>
-      </c>
-      <c r="D48" s="57"/>
-      <c r="E48" s="57"/>
-      <c r="F48" s="57"/>
-      <c r="G48" s="58"/>
-    </row>
-    <row r="49" spans="1:7" ht="42.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="59" t="s">
+      <c r="B48" s="66"/>
+      <c r="C48" s="69" t="s">
+        <v>29</v>
+      </c>
+      <c r="D48" s="70"/>
+      <c r="E48" s="70"/>
+      <c r="F48" s="70"/>
+      <c r="G48" s="71"/>
+    </row>
+    <row r="49" spans="1:7" ht="42.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="65" t="s">
         <v>16</v>
       </c>
-      <c r="B49" s="60"/>
-      <c r="C49" s="61"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="63" t="s">
+      <c r="B49" s="67"/>
+      <c r="C49" s="72"/>
+      <c r="D49" s="73"/>
+      <c r="E49" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="F49" s="63"/>
-      <c r="G49" s="64"/>
-    </row>
-    <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="59" t="s">
+      <c r="F49" s="64"/>
+      <c r="G49" s="68"/>
+    </row>
+    <row r="50" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="B50" s="60"/>
-      <c r="C50" s="65" t="s">
-        <v>29</v>
-      </c>
-      <c r="D50" s="66"/>
-      <c r="E50" s="67" t="s">
+      <c r="B50" s="67"/>
+      <c r="C50" s="74"/>
+      <c r="D50" s="75"/>
+      <c r="E50" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="F50" s="67"/>
-      <c r="G50" s="68"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="49"/>
     </row>
     <row r="51" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="47" t="s">
+      <c r="A51" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="B51" s="48"/>
-      <c r="C51" s="49" t="s">
-        <v>30</v>
-      </c>
-      <c r="D51" s="50"/>
-      <c r="E51" s="51" t="s">
+      <c r="B51" s="67"/>
+      <c r="C51" s="77"/>
+      <c r="D51" s="75"/>
+      <c r="E51" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="F51" s="51"/>
-      <c r="G51" s="52"/>
+      <c r="F51" s="61"/>
+      <c r="G51" s="62"/>
     </row>
   </sheetData>
-  <mergeCells count="96">
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:G4"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C29:D29"/>
+  <mergeCells count="94">
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C48:G48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="E49:G49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C43:D43"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="E31:F31"/>
     <mergeCell ref="C37:D37"/>
@@ -2378,34 +2245,58 @@
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="C48:G48"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="E49:G49"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:G4"/>
+    <mergeCell ref="B4:D4"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>

</xml_diff>